<commit_message>
March 9 2023 with LV_TMTT0011419
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0009535_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTabLightningView.xlsx
+++ b/TestData/LV_TMTT0009535_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTabLightningView.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112389AE-618A-4B55-B47F-F0CA0237601B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE78547-8262-436E-A908-D9B9742F1676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="5" r:id="rId1"/>
+    <sheet name="User" sheetId="5" r:id="rId1"/>
     <sheet name="AppName" sheetId="12" r:id="rId2"/>
     <sheet name="ModuleName" sheetId="13" r:id="rId3"/>
     <sheet name="SummaryLogs" sheetId="7" r:id="rId4"/>

</xml_diff>

<commit_message>
T2274-75 and db referesh TRM changes June 28 24
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0009535_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTabLightningView.xlsx
+++ b/TestData/LV_TMTT0009535_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTabLightningView.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC04086-6909-49F0-8B7A-18410298A8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F26CFFE-6C3B-40B4-A375-4A39097B8DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -152,12 +152,6 @@
     <t>DRC - Original</t>
   </si>
   <si>
-    <t>Rahimeh Bahrampourian</t>
-  </si>
-  <si>
-    <t>Salesforce Administrator</t>
-  </si>
-  <si>
     <t>Ashley Choi</t>
   </si>
   <si>
@@ -186,6 +180,12 @@
   </si>
   <si>
     <t>Time Record Manager</t>
+  </si>
+  <si>
+    <t>Nicole Bicho</t>
+  </si>
+  <si>
+    <t>Executive Administrator</t>
   </si>
 </sst>
 </file>
@@ -522,33 +522,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -560,19 +560,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC66A711-D13E-4D12-977A-ACBEF04C87E7}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -583,19 +583,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81CF81A0-141C-44BF-BC82-4486379D0B0F}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -606,17 +606,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -636,7 +636,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -656,7 +656,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -676,7 +676,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -725,16 +725,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -751,7 +751,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -768,7 +768,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -785,7 +785,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -802,7 +802,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -828,14 +828,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -843,7 +843,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -851,7 +851,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -859,7 +859,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -867,7 +867,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -884,14 +884,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -899,21 +899,21 @@
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -924,7 +924,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -935,7 +935,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>23</v>
       </c>

</xml_diff>